<commit_message>
CONSOLIDACIÓN DEL ARCHIVO FINAL DE GENERACIÓN DE DATA DE FUNEL SPRINT 4
</commit_message>
<xml_diff>
--- a/Grouped_sales_data.xlsx
+++ b/Grouped_sales_data.xlsx
@@ -519,7 +519,7 @@
         <v>17</v>
       </c>
       <c r="D4">
-        <v>229483300</v>
+        <v>229445350</v>
       </c>
       <c r="E4">
         <v>12000</v>
@@ -528,10 +528,10 @@
         <v>250</v>
       </c>
       <c r="G4">
-        <v>956.8941001830532</v>
+        <v>955.3296776503702</v>
       </c>
       <c r="H4">
-        <v>3397250.8</v>
+        <v>3400064.6</v>
       </c>
       <c r="I4">
         <v>185</v>
@@ -540,10 +540,10 @@
         <v>5.3</v>
       </c>
       <c r="K4">
-        <v>14.23552374646967</v>
+        <v>14.22841444072932</v>
       </c>
       <c r="L4">
-        <v>8091852.5</v>
+        <v>7948420</v>
       </c>
       <c r="M4">
         <v>2400</v>
@@ -552,7 +552,7 @@
         <v>0</v>
       </c>
       <c r="O4">
-        <v>33.74121740798346</v>
+        <v>33.09442320983953</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -566,7 +566,7 @@
         <v>17</v>
       </c>
       <c r="D5">
-        <v>142503350</v>
+        <v>142730750</v>
       </c>
       <c r="E5">
         <v>12000</v>
@@ -575,10 +575,10 @@
         <v>250</v>
       </c>
       <c r="G5">
-        <v>952.7726704420093</v>
+        <v>953.6873087356844</v>
       </c>
       <c r="H5">
-        <v>2117880.4</v>
+        <v>2114960.6</v>
       </c>
       <c r="I5">
         <v>185</v>
@@ -587,10 +587,10 @@
         <v>5.3</v>
       </c>
       <c r="K5">
-        <v>14.2285729641847</v>
+        <v>14.20275464703986</v>
       </c>
       <c r="L5">
-        <v>4967345</v>
+        <v>4997270</v>
       </c>
       <c r="M5">
         <v>2400</v>
@@ -599,7 +599,7 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>33.21150387451777</v>
+        <v>33.39037297376755</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -613,7 +613,7 @@
         <v>18</v>
       </c>
       <c r="D6">
-        <v>70698880</v>
+        <v>70079920</v>
       </c>
       <c r="E6">
         <v>8000</v>
@@ -622,10 +622,10 @@
         <v>120</v>
       </c>
       <c r="G6">
-        <v>588.6667776852623</v>
+        <v>581.045684437443</v>
       </c>
       <c r="H6">
-        <v>7935341</v>
+        <v>7896281.5</v>
       </c>
       <c r="I6">
         <v>680</v>
@@ -634,10 +634,10 @@
         <v>27.5</v>
       </c>
       <c r="K6">
-        <v>66.42286991386743</v>
+        <v>65.81276618797976</v>
       </c>
       <c r="L6">
-        <v>2478894</v>
+        <v>2455278</v>
       </c>
       <c r="M6">
         <v>1600</v>
@@ -646,7 +646,7 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>20.64024979184013</v>
+        <v>20.35716773070226</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -660,7 +660,7 @@
         <v>17</v>
       </c>
       <c r="D7">
-        <v>57842450</v>
+        <v>58534400</v>
       </c>
       <c r="E7">
         <v>12000</v>
@@ -669,10 +669,10 @@
         <v>250</v>
       </c>
       <c r="G7">
-        <v>1058.920071763328</v>
+        <v>1060.867043642163</v>
       </c>
       <c r="H7">
-        <v>739963.7</v>
+        <v>746871.95</v>
       </c>
       <c r="I7">
         <v>185</v>
@@ -681,10 +681,10 @@
         <v>5.3</v>
       </c>
       <c r="K7">
-        <v>13.61654122886112</v>
+        <v>13.6010043159179</v>
       </c>
       <c r="L7">
-        <v>2036192.5</v>
+        <v>2097422.5</v>
       </c>
       <c r="M7">
         <v>2400</v>
@@ -693,7 +693,7 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>37.27651764792033</v>
+        <v>38.01331194722343</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -707,7 +707,7 @@
         <v>18</v>
       </c>
       <c r="D8">
-        <v>43887640</v>
+        <v>43933840</v>
       </c>
       <c r="E8">
         <v>8000</v>
@@ -716,10 +716,10 @@
         <v>120</v>
       </c>
       <c r="G8">
-        <v>584.1870990070016</v>
+        <v>587.4450446595711</v>
       </c>
       <c r="H8">
-        <v>4950217</v>
+        <v>4943080</v>
       </c>
       <c r="I8">
         <v>680</v>
@@ -728,10 +728,10 @@
         <v>27.5</v>
       </c>
       <c r="K8">
-        <v>66.21035243763794</v>
+        <v>66.41068357695615</v>
       </c>
       <c r="L8">
-        <v>1490964</v>
+        <v>1520186</v>
       </c>
       <c r="M8">
         <v>1600</v>
@@ -740,7 +740,7 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>19.84617842025397</v>
+        <v>20.32660319837407</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -754,7 +754,7 @@
         <v>17</v>
       </c>
       <c r="D9">
-        <v>37485500</v>
+        <v>37447450</v>
       </c>
       <c r="E9">
         <v>12000</v>
@@ -763,10 +763,10 @@
         <v>250</v>
       </c>
       <c r="G9">
-        <v>991.942312781159</v>
+        <v>991.1452543539251</v>
       </c>
       <c r="H9">
-        <v>597101.45</v>
+        <v>590738.4</v>
       </c>
       <c r="I9">
         <v>185</v>
@@ -775,10 +775,10 @@
         <v>5.3</v>
       </c>
       <c r="K9">
-        <v>15.88542753006278</v>
+        <v>15.71405314819248</v>
       </c>
       <c r="L9">
-        <v>1299445</v>
+        <v>1310125</v>
       </c>
       <c r="M9">
         <v>2400</v>
@@ -787,7 +787,7 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>34.38594866366763</v>
+        <v>34.67590386956752</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -801,7 +801,7 @@
         <v>17</v>
       </c>
       <c r="D10">
-        <v>33730050</v>
+        <v>34027350</v>
       </c>
       <c r="E10">
         <v>12000</v>
@@ -810,10 +810,10 @@
         <v>250</v>
       </c>
       <c r="G10">
-        <v>983.8710147886708</v>
+        <v>993.3252568893041</v>
       </c>
       <c r="H10">
-        <v>535569.25</v>
+        <v>533038.65</v>
       </c>
       <c r="I10">
         <v>185</v>
@@ -822,19 +822,19 @@
         <v>5.3</v>
       </c>
       <c r="K10">
-        <v>15.69341723561989</v>
+        <v>15.63667605385902</v>
       </c>
       <c r="L10">
-        <v>1194280</v>
+        <v>1175535</v>
       </c>
       <c r="M10">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="N10">
         <v>0</v>
       </c>
       <c r="O10">
-        <v>34.83592451069043</v>
+        <v>34.31617818776273</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -848,7 +848,7 @@
         <v>17</v>
       </c>
       <c r="D11">
-        <v>28584950</v>
+        <v>29248900</v>
       </c>
       <c r="E11">
         <v>12000</v>
@@ -857,10 +857,10 @@
         <v>250</v>
       </c>
       <c r="G11">
-        <v>1062.361095625674</v>
+        <v>1061.011354155331</v>
       </c>
       <c r="H11">
-        <v>360817.3</v>
+        <v>373190</v>
       </c>
       <c r="I11">
         <v>185</v>
@@ -869,10 +869,10 @@
         <v>5.3</v>
       </c>
       <c r="K11">
-        <v>13.47338685586258</v>
+        <v>13.60517681370762</v>
       </c>
       <c r="L11">
-        <v>1000865</v>
+        <v>1014592.5</v>
       </c>
       <c r="M11">
         <v>2400</v>
@@ -881,7 +881,7 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>37.19719775523098</v>
+        <v>36.80460333006856</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -895,7 +895,7 @@
         <v>17</v>
       </c>
       <c r="D12">
-        <v>26352400</v>
+        <v>26332600</v>
       </c>
       <c r="E12">
         <v>12000</v>
@@ -904,10 +904,10 @@
         <v>250</v>
       </c>
       <c r="G12">
-        <v>996.1970286923978</v>
+        <v>999.8708991494532</v>
       </c>
       <c r="H12">
-        <v>417221.75</v>
+        <v>415502.1</v>
       </c>
       <c r="I12">
         <v>185</v>
@@ -916,10 +916,10 @@
         <v>5.3</v>
       </c>
       <c r="K12">
-        <v>15.84466618562965</v>
+        <v>15.8630970106517</v>
       </c>
       <c r="L12">
-        <v>922392.5</v>
+        <v>933737.5</v>
       </c>
       <c r="M12">
         <v>2400</v>
@@ -928,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>34.86910747363248</v>
+        <v>35.45479571688943</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -942,7 +942,7 @@
         <v>19</v>
       </c>
       <c r="D13">
-        <v>19842605</v>
+        <v>19808755</v>
       </c>
       <c r="E13">
         <v>1500</v>
@@ -951,10 +951,10 @@
         <v>35</v>
       </c>
       <c r="G13">
-        <v>123.6199248658987</v>
+        <v>123.7869243796204</v>
       </c>
       <c r="H13">
-        <v>2284878.7</v>
+        <v>2280922.3</v>
       </c>
       <c r="I13">
         <v>155</v>
@@ -963,10 +963,10 @@
         <v>5.9</v>
       </c>
       <c r="K13">
-        <v>14.30481005208855</v>
+        <v>14.32632150842901</v>
       </c>
       <c r="L13">
-        <v>696447.5</v>
+        <v>692503.75</v>
       </c>
       <c r="M13">
         <v>300</v>
@@ -975,7 +975,7 @@
         <v>0</v>
       </c>
       <c r="O13">
-        <v>4.338885323930149</v>
+        <v>4.327526355586384</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -989,7 +989,7 @@
         <v>17</v>
       </c>
       <c r="D14">
-        <v>17756400</v>
+        <v>17550850</v>
       </c>
       <c r="E14">
         <v>12000</v>
@@ -998,10 +998,10 @@
         <v>250</v>
       </c>
       <c r="G14">
-        <v>958.768898488121</v>
+        <v>966.9889807162534</v>
       </c>
       <c r="H14">
-        <v>264007.15</v>
+        <v>255463.55</v>
       </c>
       <c r="I14">
         <v>185</v>
@@ -1010,19 +1010,19 @@
         <v>5.3</v>
       </c>
       <c r="K14">
-        <v>14.33341386611651</v>
+        <v>14.15859613146372</v>
       </c>
       <c r="L14">
-        <v>622852.5</v>
+        <v>606722.5</v>
       </c>
       <c r="M14">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="N14">
         <v>0</v>
       </c>
       <c r="O14">
-        <v>33.6313444924406</v>
+        <v>33.42823691460055</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -1036,7 +1036,7 @@
         <v>20</v>
       </c>
       <c r="D15">
-        <v>17023665</v>
+        <v>16889520</v>
       </c>
       <c r="E15">
         <v>1200</v>
@@ -1045,10 +1045,10 @@
         <v>20</v>
       </c>
       <c r="G15">
-        <v>106.3786251241962</v>
+        <v>105.6466584932569</v>
       </c>
       <c r="H15">
-        <v>1003075.4</v>
+        <v>1000835.35</v>
       </c>
       <c r="I15">
         <v>17</v>
@@ -1057,10 +1057,10 @@
         <v>5.3</v>
       </c>
       <c r="K15">
-        <v>6.299933425449065</v>
+        <v>6.292227098120823</v>
       </c>
       <c r="L15">
-        <v>592422.75</v>
+        <v>588268</v>
       </c>
       <c r="M15">
         <v>240</v>
@@ -1069,7 +1069,7 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>3.701971205219054</v>
+        <v>3.679710761378137</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -1083,7 +1083,7 @@
         <v>21</v>
       </c>
       <c r="D16">
-        <v>14525709</v>
+        <v>14639715</v>
       </c>
       <c r="E16">
         <v>1500</v>
@@ -1092,10 +1092,10 @@
         <v>25.5</v>
       </c>
       <c r="G16">
-        <v>121.0213537066969</v>
+        <v>121.2589558605495</v>
       </c>
       <c r="H16">
-        <v>756868.25</v>
+        <v>761912.1</v>
       </c>
       <c r="I16">
         <v>23</v>
@@ -1104,10 +1104,10 @@
         <v>5.15</v>
       </c>
       <c r="K16">
-        <v>6.339514109340056</v>
+        <v>6.341974229635919</v>
       </c>
       <c r="L16">
-        <v>507584.3</v>
+        <v>510561.075</v>
       </c>
       <c r="M16">
         <v>300</v>
@@ -1116,7 +1116,7 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>4.228952893539733</v>
+        <v>4.228914487579826</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -1130,7 +1130,7 @@
         <v>19</v>
       </c>
       <c r="D17">
-        <v>12381265</v>
+        <v>12399095</v>
       </c>
       <c r="E17">
         <v>1500</v>
@@ -1139,10 +1139,10 @@
         <v>35</v>
       </c>
       <c r="G17">
-        <v>123.9365865865866</v>
+        <v>124.04925314898</v>
       </c>
       <c r="H17">
-        <v>1425391.8</v>
+        <v>1425478.1</v>
       </c>
       <c r="I17">
         <v>155</v>
@@ -1151,10 +1151,10 @@
         <v>5.9</v>
       </c>
       <c r="K17">
-        <v>14.33966922194725</v>
+        <v>14.33433656795214</v>
       </c>
       <c r="L17">
-        <v>434634.5</v>
+        <v>428642.75</v>
       </c>
       <c r="M17">
         <v>300</v>
@@ -1163,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>4.350695695695696</v>
+        <v>4.288443068242074</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -1177,7 +1177,7 @@
         <v>20</v>
       </c>
       <c r="D18">
-        <v>10597265</v>
+        <v>10535325</v>
       </c>
       <c r="E18">
         <v>1200</v>
@@ -1186,10 +1186,10 @@
         <v>20</v>
       </c>
       <c r="G18">
-        <v>106.0182378422722</v>
+        <v>105.6458891128426</v>
       </c>
       <c r="H18">
-        <v>626119.15</v>
+        <v>624370.85</v>
       </c>
       <c r="I18">
         <v>17</v>
@@ -1198,10 +1198,10 @@
         <v>5.3</v>
       </c>
       <c r="K18">
-        <v>6.29702155263449</v>
+        <v>6.293553443270704</v>
       </c>
       <c r="L18">
-        <v>368313.25</v>
+        <v>368094.25</v>
       </c>
       <c r="M18">
         <v>240</v>
@@ -1210,7 +1210,7 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>3.68471692827916</v>
+        <v>3.691167032680525</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1224,7 +1224,7 @@
         <v>21</v>
       </c>
       <c r="D19">
-        <v>9044107</v>
+        <v>9174809</v>
       </c>
       <c r="E19">
         <v>1500</v>
@@ -1233,10 +1233,10 @@
         <v>25.5</v>
       </c>
       <c r="G19">
-        <v>120.8685082725256</v>
+        <v>121.8159114144217</v>
       </c>
       <c r="H19">
-        <v>471903.1</v>
+        <v>475993.75</v>
       </c>
       <c r="I19">
         <v>23</v>
@@ -1245,10 +1245,10 @@
         <v>5.15</v>
       </c>
       <c r="K19">
-        <v>6.337502350192044</v>
+        <v>6.349461755996051</v>
       </c>
       <c r="L19">
-        <v>313965.925</v>
+        <v>326480</v>
       </c>
       <c r="M19">
         <v>300</v>
@@ -1257,7 +1257,7 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>4.195946930211424</v>
+        <v>4.334745143858624</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1268,43 +1268,43 @@
         <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D20">
-        <v>8774080</v>
+        <v>8771740</v>
       </c>
       <c r="E20">
-        <v>8000</v>
+        <v>1500</v>
       </c>
       <c r="F20">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="G20">
-        <v>488.2083240596484</v>
+        <v>122.0161357629712</v>
       </c>
       <c r="H20">
-        <v>1019678</v>
+        <v>1003436.8</v>
       </c>
       <c r="I20">
-        <v>680</v>
+        <v>155</v>
       </c>
       <c r="J20">
-        <v>27.5</v>
+        <v>5.9</v>
       </c>
       <c r="K20">
-        <v>56.98753702565249</v>
+        <v>14.02388193202147</v>
       </c>
       <c r="L20">
-        <v>305968</v>
+        <v>306813</v>
       </c>
       <c r="M20">
-        <v>1600</v>
+        <v>300</v>
       </c>
       <c r="N20">
         <v>0</v>
       </c>
       <c r="O20">
-        <v>17.02470509681727</v>
+        <v>4.267811934900543</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -1315,43 +1315,43 @@
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D21">
-        <v>8731150</v>
+        <v>8726840</v>
       </c>
       <c r="E21">
-        <v>1500</v>
+        <v>8000</v>
       </c>
       <c r="F21">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="G21">
-        <v>121.0809873803911</v>
+        <v>491.2101767420916</v>
       </c>
       <c r="H21">
-        <v>998913.1</v>
+        <v>1011286</v>
       </c>
       <c r="I21">
-        <v>155</v>
+        <v>680</v>
       </c>
       <c r="J21">
-        <v>5.9</v>
+        <v>27.5</v>
       </c>
       <c r="K21">
-        <v>13.92329811552186</v>
+        <v>57.14771699819168</v>
       </c>
       <c r="L21">
-        <v>304993</v>
+        <v>306092</v>
       </c>
       <c r="M21">
-        <v>300</v>
+        <v>1600</v>
       </c>
       <c r="N21">
         <v>0</v>
       </c>
       <c r="O21">
-        <v>4.229552073221467</v>
+        <v>17.22908927164246</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -1365,7 +1365,7 @@
         <v>18</v>
       </c>
       <c r="D22">
-        <v>8047080</v>
+        <v>7993640</v>
       </c>
       <c r="E22">
         <v>8000</v>
@@ -1374,10 +1374,10 @@
         <v>120</v>
       </c>
       <c r="G22">
-        <v>492.3869546594872</v>
+        <v>492.765380347676</v>
       </c>
       <c r="H22">
-        <v>934669.5</v>
+        <v>930575.5</v>
       </c>
       <c r="I22">
         <v>680</v>
@@ -1386,10 +1386,10 @@
         <v>27.5</v>
       </c>
       <c r="K22">
-        <v>57.52520310192023</v>
+        <v>57.61720636493096</v>
       </c>
       <c r="L22">
-        <v>274418</v>
+        <v>271010</v>
       </c>
       <c r="M22">
         <v>1600</v>
@@ -1398,7 +1398,7 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <v>16.79116441289849</v>
+        <v>16.70632474417458</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -1412,7 +1412,7 @@
         <v>19</v>
       </c>
       <c r="D23">
-        <v>7893935</v>
+        <v>7922850</v>
       </c>
       <c r="E23">
         <v>1500</v>
@@ -1421,10 +1421,10 @@
         <v>35</v>
       </c>
       <c r="G23">
-        <v>121.7410783134388</v>
+        <v>121.860003691399</v>
       </c>
       <c r="H23">
-        <v>902367.2000000001</v>
+        <v>907902.4</v>
       </c>
       <c r="I23">
         <v>155</v>
@@ -1433,10 +1433,10 @@
         <v>5.9</v>
       </c>
       <c r="K23">
-        <v>13.98346841053137</v>
+        <v>14.03900417504252</v>
       </c>
       <c r="L23">
-        <v>276509.75</v>
+        <v>278364.5</v>
       </c>
       <c r="M23">
         <v>300</v>
@@ -1445,7 +1445,7 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>4.2643618333796</v>
+        <v>4.281476867232681</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -1453,46 +1453,46 @@
         <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C24" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D24">
-        <v>6228305</v>
+        <v>6288880</v>
       </c>
       <c r="E24">
-        <v>1200</v>
+        <v>8000</v>
       </c>
       <c r="F24">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="G24">
-        <v>94.14430823646779</v>
+        <v>502.6680521141396</v>
       </c>
       <c r="H24">
-        <v>402491.05</v>
+        <v>724510.5</v>
       </c>
       <c r="I24">
-        <v>17</v>
+        <v>680</v>
       </c>
       <c r="J24">
-        <v>5.3</v>
+        <v>27.5</v>
       </c>
       <c r="K24">
-        <v>6.112890512279209</v>
+        <v>58.15157717312786</v>
       </c>
       <c r="L24">
-        <v>217678.5</v>
+        <v>215984</v>
       </c>
       <c r="M24">
-        <v>240</v>
+        <v>800</v>
       </c>
       <c r="N24">
         <v>0</v>
       </c>
       <c r="O24">
-        <v>3.290332088819021</v>
+        <v>17.26352809527616</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -1500,46 +1500,46 @@
         <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D25">
-        <v>6223920</v>
+        <v>6242625</v>
       </c>
       <c r="E25">
-        <v>8000</v>
+        <v>1200</v>
       </c>
       <c r="F25">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="G25">
-        <v>498.1128451380552</v>
+        <v>95.05908239557796</v>
       </c>
       <c r="H25">
-        <v>721864</v>
+        <v>400228.95</v>
       </c>
       <c r="I25">
-        <v>680</v>
+        <v>17</v>
       </c>
       <c r="J25">
-        <v>27.5</v>
+        <v>5.3</v>
       </c>
       <c r="K25">
-        <v>58.02765273311897</v>
+        <v>6.123079217918121</v>
       </c>
       <c r="L25">
-        <v>218610</v>
+        <v>217661.75</v>
       </c>
       <c r="M25">
-        <v>1600</v>
+        <v>240</v>
       </c>
       <c r="N25">
         <v>0</v>
       </c>
       <c r="O25">
-        <v>17.49579831932773</v>
+        <v>3.314427220538746</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -1553,7 +1553,7 @@
         <v>19</v>
       </c>
       <c r="D26">
-        <v>6103475</v>
+        <v>6071395</v>
       </c>
       <c r="E26">
         <v>1500</v>
@@ -1562,10 +1562,10 @@
         <v>35</v>
       </c>
       <c r="G26">
-        <v>121.840439972851</v>
+        <v>120.6365243999364</v>
       </c>
       <c r="H26">
-        <v>697164.7000000001</v>
+        <v>694805.4</v>
       </c>
       <c r="I26">
         <v>155</v>
@@ -1574,10 +1574,10 @@
         <v>5.9</v>
       </c>
       <c r="K26">
-        <v>13.98861711946707</v>
+        <v>13.88416761585037</v>
       </c>
       <c r="L26">
-        <v>216904</v>
+        <v>214185.75</v>
       </c>
       <c r="M26">
         <v>300</v>
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <v>4.329939713338923</v>
+        <v>4.255796971864569</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -1600,7 +1600,7 @@
         <v>20</v>
       </c>
       <c r="D27">
-        <v>5618155</v>
+        <v>5639005</v>
       </c>
       <c r="E27">
         <v>1200</v>
@@ -1609,10 +1609,10 @@
         <v>20</v>
       </c>
       <c r="G27">
-        <v>93.91295989836685</v>
+        <v>94.63323152312546</v>
       </c>
       <c r="H27">
-        <v>363723.7</v>
+        <v>362700.45</v>
       </c>
       <c r="I27">
         <v>17</v>
@@ -1621,10 +1621,10 @@
         <v>5.3</v>
       </c>
       <c r="K27">
-        <v>6.110435951280975</v>
+        <v>6.117190346083789</v>
       </c>
       <c r="L27">
-        <v>195038</v>
+        <v>199652.75</v>
       </c>
       <c r="M27">
         <v>240</v>
@@ -1633,7 +1633,7 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>3.260251074001638</v>
+        <v>3.350552963683963</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -1647,7 +1647,7 @@
         <v>18</v>
       </c>
       <c r="D28">
-        <v>5394400</v>
+        <v>5339080</v>
       </c>
       <c r="E28">
         <v>8000</v>
@@ -1656,10 +1656,10 @@
         <v>120</v>
       </c>
       <c r="G28">
-        <v>590.0032811987313</v>
+        <v>589.3674798542886</v>
       </c>
       <c r="H28">
-        <v>607782</v>
+        <v>599072</v>
       </c>
       <c r="I28">
         <v>680</v>
@@ -1668,19 +1668,19 @@
         <v>27.5</v>
       </c>
       <c r="K28">
-        <v>66.81860158311346</v>
+        <v>66.42332852866171</v>
       </c>
       <c r="L28">
-        <v>187824</v>
+        <v>185322</v>
       </c>
       <c r="M28">
-        <v>1600</v>
+        <v>800</v>
       </c>
       <c r="N28">
         <v>0</v>
       </c>
       <c r="O28">
-        <v>20.54292901673411</v>
+        <v>20.45722485925599</v>
       </c>
     </row>
     <row r="29" spans="1:15">
@@ -1694,7 +1694,7 @@
         <v>20</v>
       </c>
       <c r="D29">
-        <v>4375505</v>
+        <v>4294610</v>
       </c>
       <c r="E29">
         <v>1200</v>
@@ -1703,10 +1703,10 @@
         <v>20</v>
       </c>
       <c r="G29">
-        <v>94.96277888705617</v>
+        <v>94.05010621290761</v>
       </c>
       <c r="H29">
-        <v>280401.7</v>
+        <v>277590.35</v>
       </c>
       <c r="I29">
         <v>17</v>
@@ -1715,10 +1715,10 @@
         <v>5.3</v>
       </c>
       <c r="K29">
-        <v>6.119902658343882</v>
+        <v>6.111094355406833</v>
       </c>
       <c r="L29">
-        <v>155420</v>
+        <v>148822</v>
       </c>
       <c r="M29">
         <v>240</v>
@@ -1727,7 +1727,7 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>3.373122666898168</v>
+        <v>3.259137594989379</v>
       </c>
     </row>
     <row r="30" spans="1:15">
@@ -1741,7 +1741,7 @@
         <v>18</v>
       </c>
       <c r="D30">
-        <v>1855120</v>
+        <v>1814400</v>
       </c>
       <c r="E30">
         <v>8000</v>
@@ -1750,10 +1750,10 @@
         <v>120</v>
       </c>
       <c r="G30">
-        <v>383.2892561983471</v>
+        <v>376.7441860465116</v>
       </c>
       <c r="H30">
-        <v>225941</v>
+        <v>222574.5</v>
       </c>
       <c r="I30">
         <v>680</v>
@@ -1762,19 +1762,19 @@
         <v>27.5</v>
       </c>
       <c r="K30">
-        <v>46.91465946843854</v>
+        <v>46.4859022556391</v>
       </c>
       <c r="L30">
-        <v>66954</v>
+        <v>63756</v>
       </c>
       <c r="M30">
-        <v>800</v>
+        <v>640</v>
       </c>
       <c r="N30">
         <v>0</v>
       </c>
       <c r="O30">
-        <v>13.83347107438017</v>
+        <v>13.23837209302326</v>
       </c>
     </row>
     <row r="31" spans="1:15">
@@ -1788,7 +1788,7 @@
         <v>21</v>
       </c>
       <c r="D31">
-        <v>1666771.5</v>
+        <v>1682928</v>
       </c>
       <c r="E31">
         <v>1500</v>
@@ -1797,10 +1797,10 @@
         <v>25.5</v>
       </c>
       <c r="G31">
-        <v>161.0718496327793</v>
+        <v>160.7534626038781</v>
       </c>
       <c r="H31">
-        <v>70343.75</v>
+        <v>71149.10000000001</v>
       </c>
       <c r="I31">
         <v>23</v>
@@ -1809,10 +1809,10 @@
         <v>5.15</v>
       </c>
       <c r="K31">
-        <v>6.837456259720062</v>
+        <v>6.832062608027655</v>
       </c>
       <c r="L31">
-        <v>58258.875</v>
+        <v>59369.325</v>
       </c>
       <c r="M31">
         <v>300</v>
@@ -1821,7 +1821,7 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>5.629964727483571</v>
+        <v>5.670964275479988</v>
       </c>
     </row>
     <row r="32" spans="1:15">
@@ -1835,7 +1835,7 @@
         <v>19</v>
       </c>
       <c r="D32">
-        <v>1516875</v>
+        <v>1483515</v>
       </c>
       <c r="E32">
         <v>1500</v>
@@ -1844,10 +1844,10 @@
         <v>35</v>
       </c>
       <c r="G32">
-        <v>124.4156003937008</v>
+        <v>123.2155315614618</v>
       </c>
       <c r="H32">
-        <v>174086.7</v>
+        <v>171093.8</v>
       </c>
       <c r="I32">
         <v>155</v>
@@ -1856,19 +1856,19 @@
         <v>5.9</v>
       </c>
       <c r="K32">
-        <v>14.34228868017795</v>
+        <v>14.27447021525112</v>
       </c>
       <c r="L32">
-        <v>53378.5</v>
+        <v>52031.25</v>
       </c>
       <c r="M32">
-        <v>170</v>
+        <v>300</v>
       </c>
       <c r="N32">
         <v>0</v>
       </c>
       <c r="O32">
-        <v>4.37815780839895</v>
+        <v>4.321532392026578</v>
       </c>
     </row>
     <row r="33" spans="1:15">
@@ -1882,7 +1882,7 @@
         <v>20</v>
       </c>
       <c r="D33">
-        <v>1288850</v>
+        <v>1273620</v>
       </c>
       <c r="E33">
         <v>1200</v>
@@ -1891,10 +1891,10 @@
         <v>20</v>
       </c>
       <c r="G33">
-        <v>105.9038619556286</v>
+        <v>106.9549882431978</v>
       </c>
       <c r="H33">
-        <v>76315.8</v>
+        <v>74764.64999999999</v>
       </c>
       <c r="I33">
         <v>17</v>
@@ -1903,19 +1903,19 @@
         <v>5.3</v>
       </c>
       <c r="K33">
-        <v>6.298242139143353</v>
+        <v>6.30765628954695</v>
       </c>
       <c r="L33">
-        <v>46095.25</v>
+        <v>44443</v>
       </c>
       <c r="M33">
-        <v>120</v>
+        <v>170</v>
       </c>
       <c r="N33">
         <v>0</v>
       </c>
       <c r="O33">
-        <v>3.787612982744454</v>
+        <v>3.732196842458851</v>
       </c>
     </row>
     <row r="34" spans="1:15">
@@ -1929,7 +1929,7 @@
         <v>21</v>
       </c>
       <c r="D34">
-        <v>1092294</v>
+        <v>1077665</v>
       </c>
       <c r="E34">
         <v>1500</v>
@@ -1938,10 +1938,10 @@
         <v>25.5</v>
       </c>
       <c r="G34">
-        <v>118.5086253661712</v>
+        <v>120.3288298347477</v>
       </c>
       <c r="H34">
-        <v>57816.1</v>
+        <v>56390.8</v>
       </c>
       <c r="I34">
         <v>23</v>
@@ -1950,10 +1950,10 @@
         <v>5.15</v>
       </c>
       <c r="K34">
-        <v>6.309046268005238</v>
+        <v>6.333909918005166</v>
       </c>
       <c r="L34">
-        <v>37038.275</v>
+        <v>38744.425</v>
       </c>
       <c r="M34">
         <v>300</v>
@@ -1962,7 +1962,7 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>4.018474015406315</v>
+        <v>4.326085864225101</v>
       </c>
     </row>
     <row r="35" spans="1:15">
@@ -1976,7 +1976,7 @@
         <v>18</v>
       </c>
       <c r="D35">
-        <v>929440</v>
+        <v>946080</v>
       </c>
       <c r="E35">
         <v>8000</v>
@@ -1985,10 +1985,10 @@
         <v>120</v>
       </c>
       <c r="G35">
-        <v>389.7023060796646</v>
+        <v>394.6933667083855</v>
       </c>
       <c r="H35">
-        <v>112431.5</v>
+        <v>113783</v>
       </c>
       <c r="I35">
         <v>680</v>
@@ -1997,19 +1997,19 @@
         <v>27.5</v>
       </c>
       <c r="K35">
-        <v>47.3595197978096</v>
+        <v>47.68776194467728</v>
       </c>
       <c r="L35">
-        <v>36394</v>
+        <v>34004</v>
       </c>
       <c r="M35">
-        <v>480</v>
+        <v>1600</v>
       </c>
       <c r="N35">
         <v>0</v>
       </c>
       <c r="O35">
-        <v>15.25953878406709</v>
+        <v>14.18606591572799</v>
       </c>
     </row>
     <row r="36" spans="1:15">
@@ -2023,7 +2023,7 @@
         <v>21</v>
       </c>
       <c r="D36">
-        <v>827383.5</v>
+        <v>846228</v>
       </c>
       <c r="E36">
         <v>1500</v>
@@ -2032,10 +2032,10 @@
         <v>25.5</v>
       </c>
       <c r="G36">
-        <v>162.2638752696607</v>
+        <v>161.7717453641751</v>
       </c>
       <c r="H36">
-        <v>34754</v>
+        <v>35641.75</v>
       </c>
       <c r="I36">
         <v>23</v>
@@ -2044,10 +2044,10 @@
         <v>5.15</v>
       </c>
       <c r="K36">
-        <v>6.853480575823309</v>
+        <v>6.84891429669485</v>
       </c>
       <c r="L36">
-        <v>28744.95</v>
+        <v>29161.125</v>
       </c>
       <c r="M36">
         <v>300</v>
@@ -2056,7 +2056,7 @@
         <v>0</v>
       </c>
       <c r="O36">
-        <v>5.637370072563248</v>
+        <v>5.574675014337603</v>
       </c>
     </row>
     <row r="37" spans="1:15">
@@ -2070,7 +2070,7 @@
         <v>20</v>
       </c>
       <c r="D37">
-        <v>813720</v>
+        <v>803980</v>
       </c>
       <c r="E37">
         <v>1200</v>
@@ -2079,10 +2079,10 @@
         <v>20</v>
       </c>
       <c r="G37">
-        <v>144.3021812378081</v>
+        <v>143.0314890588863</v>
       </c>
       <c r="H37">
-        <v>36429.1</v>
+        <v>36260.8</v>
       </c>
       <c r="I37">
         <v>17</v>
@@ -2091,10 +2091,10 @@
         <v>5.3</v>
       </c>
       <c r="K37">
-        <v>6.491286528866714</v>
+        <v>6.475142857142858</v>
       </c>
       <c r="L37">
-        <v>27564</v>
+        <v>28003</v>
       </c>
       <c r="M37">
         <v>240</v>
@@ -2103,7 +2103,7 @@
         <v>0</v>
       </c>
       <c r="O37">
-        <v>4.888100727079269</v>
+        <v>4.981853762675681</v>
       </c>
     </row>
     <row r="38" spans="1:15">
@@ -2117,7 +2117,7 @@
         <v>21</v>
       </c>
       <c r="D38">
-        <v>629404.5</v>
+        <v>631072.5</v>
       </c>
       <c r="E38">
         <v>1500</v>
@@ -2126,10 +2126,10 @@
         <v>25.5</v>
       </c>
       <c r="G38">
-        <v>104.6913672654691</v>
+        <v>105.6188284518828</v>
       </c>
       <c r="H38">
-        <v>36414.5</v>
+        <v>36233.35</v>
       </c>
       <c r="I38">
         <v>23</v>
@@ -2138,19 +2138,19 @@
         <v>5.15</v>
       </c>
       <c r="K38">
-        <v>6.095497154335454</v>
+        <v>6.100917662906213</v>
       </c>
       <c r="L38">
-        <v>20418</v>
+        <v>21501.525</v>
       </c>
       <c r="M38">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="N38">
         <v>0</v>
       </c>
       <c r="O38">
-        <v>3.396207584830339</v>
+        <v>3.598581589958159</v>
       </c>
     </row>
     <row r="39" spans="1:15">
@@ -2158,37 +2158,37 @@
         <v>35</v>
       </c>
       <c r="B39" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C39" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D39">
-        <v>560226</v>
+        <v>555110</v>
       </c>
       <c r="E39">
         <v>1500</v>
       </c>
       <c r="F39">
-        <v>25.5</v>
+        <v>35</v>
       </c>
       <c r="G39">
-        <v>103.8802150936399</v>
+        <v>116.8898715519057</v>
       </c>
       <c r="H39">
-        <v>32628.8</v>
+        <v>62047</v>
       </c>
       <c r="I39">
-        <v>23</v>
+        <v>155</v>
       </c>
       <c r="J39">
-        <v>5.15</v>
+        <v>5.9</v>
       </c>
       <c r="K39">
-        <v>6.078390461997019</v>
+        <v>13.15112335735481</v>
       </c>
       <c r="L39">
-        <v>21738.975</v>
+        <v>19859.5</v>
       </c>
       <c r="M39">
         <v>150</v>
@@ -2197,7 +2197,7 @@
         <v>0</v>
       </c>
       <c r="O39">
-        <v>4.030961431485259</v>
+        <v>4.181827753211202</v>
       </c>
     </row>
     <row r="40" spans="1:15">
@@ -2205,46 +2205,46 @@
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C40" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D40">
-        <v>554290</v>
+        <v>553774.5</v>
       </c>
       <c r="E40">
         <v>1500</v>
       </c>
       <c r="F40">
-        <v>35</v>
+        <v>25.5</v>
       </c>
       <c r="G40">
-        <v>113.8172484599589</v>
+        <v>103.7030898876404</v>
       </c>
       <c r="H40">
-        <v>62886.5</v>
+        <v>32435.75</v>
       </c>
       <c r="I40">
-        <v>155</v>
+        <v>23</v>
       </c>
       <c r="J40">
-        <v>5.9</v>
+        <v>5.15</v>
       </c>
       <c r="K40">
-        <v>12.96896267271602</v>
+        <v>6.086648526928129</v>
       </c>
       <c r="L40">
-        <v>19116</v>
+        <v>19034.025</v>
       </c>
       <c r="M40">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="N40">
         <v>0</v>
       </c>
       <c r="O40">
-        <v>3.925256673511293</v>
+        <v>3.564424157303371</v>
       </c>
     </row>
     <row r="41" spans="1:15">
@@ -2258,7 +2258,7 @@
         <v>21</v>
       </c>
       <c r="D41">
-        <v>449196</v>
+        <v>434196</v>
       </c>
       <c r="E41">
         <v>1500</v>
@@ -2267,10 +2267,10 @@
         <v>25.5</v>
       </c>
       <c r="G41">
-        <v>108.0577339427472</v>
+        <v>102.3805706201368</v>
       </c>
       <c r="H41">
-        <v>25353.35</v>
+        <v>25616.4</v>
       </c>
       <c r="I41">
         <v>23</v>
@@ -2279,10 +2279,10 @@
         <v>5.15</v>
       </c>
       <c r="K41">
-        <v>6.126957467375544</v>
+        <v>6.068798862828714</v>
       </c>
       <c r="L41">
-        <v>14993.775</v>
+        <v>15781.5</v>
       </c>
       <c r="M41">
         <v>150</v>
@@ -2291,7 +2291,7 @@
         <v>0</v>
       </c>
       <c r="O41">
-        <v>3.606873947558335</v>
+        <v>3.721174251355812</v>
       </c>
     </row>
     <row r="42" spans="1:15">
@@ -2305,7 +2305,7 @@
         <v>20</v>
       </c>
       <c r="D42">
-        <v>411600</v>
+        <v>418840</v>
       </c>
       <c r="E42">
         <v>1200</v>
@@ -2314,10 +2314,10 @@
         <v>20</v>
       </c>
       <c r="G42">
-        <v>145.4931071049841</v>
+        <v>144.3280496209511</v>
       </c>
       <c r="H42">
-        <v>18327.1</v>
+        <v>18695.1</v>
       </c>
       <c r="I42">
         <v>17</v>
@@ -2326,19 +2326,19 @@
         <v>5.3</v>
       </c>
       <c r="K42">
-        <v>6.501277048598794</v>
+        <v>6.484599375650365</v>
       </c>
       <c r="L42">
-        <v>14143</v>
+        <v>13962</v>
       </c>
       <c r="M42">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="N42">
         <v>0</v>
       </c>
       <c r="O42">
-        <v>4.999293036408625</v>
+        <v>4.811164713990351</v>
       </c>
     </row>
     <row r="43" spans="1:15">
@@ -2352,7 +2352,7 @@
         <v>19</v>
       </c>
       <c r="D43">
-        <v>271740</v>
+        <v>280255</v>
       </c>
       <c r="E43">
         <v>1500</v>
@@ -2361,10 +2361,10 @@
         <v>35</v>
       </c>
       <c r="G43">
-        <v>115.5357142857143</v>
+        <v>110.9920792079208</v>
       </c>
       <c r="H43">
-        <v>31087.7</v>
+        <v>32201</v>
       </c>
       <c r="I43">
         <v>155</v>
@@ -2373,19 +2373,19 @@
         <v>5.9</v>
       </c>
       <c r="K43">
-        <v>13.26267064846416</v>
+        <v>12.77310591035303</v>
       </c>
       <c r="L43">
-        <v>9846.5</v>
+        <v>9605.25</v>
       </c>
       <c r="M43">
-        <v>170</v>
+        <v>90</v>
       </c>
       <c r="N43">
         <v>0</v>
       </c>
       <c r="O43">
-        <v>4.186437074829932</v>
+        <v>3.804059405940594</v>
       </c>
     </row>
   </sheetData>

</xml_diff>